<commit_message>
Update LP_Error_Log.xlsx with new data
</commit_message>
<xml_diff>
--- a/LP_Error_Log.xlsx
+++ b/LP_Error_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://musigma-my.sharepoint.com/personal/maria_daniels_mu-sigma_com/Documents/Documents/exel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{5EB6F39B-016E-4168-A8C8-22C4E1775C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD65717F-C4D8-4C8A-A452-759C7E7DB61F}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{5EB6F39B-016E-4168-A8C8-22C4E1775C1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{331833D1-2995-415D-8C01-C3871C4F3724}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7E36AAAB-D706-4463-8B8E-FC781FC93857}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7E36AAAB-D706-4463-8B8E-FC781FC93857}"/>
   </bookViews>
   <sheets>
     <sheet name="Error Log" sheetId="1" r:id="rId1"/>
@@ -1620,7 +1620,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDFA68B3-D723-4F82-915D-45274FA59027}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A2:Q27"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1692,7 +1691,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:16" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B3" s="10">
         <v>45846</v>
       </c>
@@ -1739,7 +1738,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="2:16" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B4" s="15">
         <v>45875</v>
       </c>
@@ -1786,7 +1785,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="2:16" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B5" s="15">
         <v>45896</v>
       </c>
@@ -1833,7 +1832,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B6" s="10" t="s">
         <v>43</v>
       </c>
@@ -1880,7 +1879,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B7" s="10" t="s">
         <v>51</v>
       </c>
@@ -1925,7 +1924,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:16" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:16" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B8" s="15">
         <v>45890</v>
       </c>
@@ -1972,7 +1971,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="2:16" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B9" s="18">
         <v>45873</v>
       </c>
@@ -2066,7 +2065,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B11" s="22">
         <v>45876</v>
       </c>
@@ -2113,7 +2112,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B12" s="23">
         <v>45833</v>
       </c>
@@ -2158,7 +2157,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B13" s="7">
         <v>45896</v>
       </c>
@@ -2205,7 +2204,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B14" s="7">
         <v>45929</v>
       </c>
@@ -2246,7 +2245,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="2:16" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B15" s="7">
         <v>45849</v>
       </c>
@@ -2293,7 +2292,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="2:16" ht="76.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:16" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="7">
         <v>45929</v>
       </c>
@@ -2340,7 +2339,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="2:16" ht="39.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:16" ht="39.5" x14ac:dyDescent="0.35">
       <c r="B17" s="7">
         <v>45966</v>
       </c>
@@ -2387,7 +2386,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="2:16" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B18" s="7">
         <v>45938</v>
       </c>
@@ -2432,7 +2431,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="2:16" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:16" ht="87" x14ac:dyDescent="0.35">
       <c r="B19" s="36">
         <v>45942</v>
       </c>
@@ -2477,7 +2476,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B20" s="40">
         <v>45788</v>
       </c>
@@ -2524,7 +2523,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="2:16" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B21" s="40">
         <v>45966</v>
       </c>
@@ -2568,7 +2567,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B22" s="40">
         <v>45978</v>
       </c>
@@ -2615,7 +2614,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="2:16" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:16" ht="87" x14ac:dyDescent="0.35">
       <c r="B23" s="40"/>
       <c r="C23" s="43"/>
       <c r="E23" s="1" t="s">
@@ -2655,7 +2654,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="24" spans="2:16" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B24" s="44" t="s">
         <v>156</v>
       </c>
@@ -2702,7 +2701,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="25" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B25" s="49">
         <v>46034</v>
       </c>
@@ -2749,7 +2748,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="26" spans="2:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B26" s="7">
         <v>46044</v>
       </c>
@@ -2797,7 +2796,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="2:16" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:16" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B27" s="7">
         <v>46072</v>
       </c>
@@ -2845,13 +2844,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:P27" xr:uid="{DDFA68B3-D723-4F82-915D-45274FA59027}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="SA"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B2:P27" xr:uid="{DDFA68B3-D723-4F82-915D-45274FA59027}"/>
   <conditionalFormatting sqref="B19">
     <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>

</xml_diff>